<commit_message>
Move Date of Service to column 5 and pin Days Until Deadline at column 10
Reorders every specialty sheet and the master to lead with Claim Status,
Notes, Primary Claim ID, Chart Number, Date of Service, Responsible Payer,
Primary Payer Name, Secondary Payer Name, Procedure Code, Days Until
Deadline. Date of Service moves up beside the chart number, and the day
count closes the pinned block at column 10.

Filing Deadline, Filing Limit and Limit Carrier follow at columns 11-13,
then the billing detail, amounts, AR age, diagnoses and reference fields as
before. Row order and all data are unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J8rYoF6JmCLXfVMQM34p4x
</commit_message>
<xml_diff>
--- a/Specialty Claims 2026-S1/2026-01 January - Specialty Claims.xlsx
+++ b/Specialty Claims 2026-S1/2026-01 January - Specialty Claims.xlsx
@@ -766,10 +766,10 @@
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
@@ -821,22 +821,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Date of Service</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Responsible Payer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Primary Payer Name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Secondary Payer Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Date of Service</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -983,22 +983,22 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
           <t>Health Choice Arizona</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Health Choice Arizona</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>01/28/2026</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -1100,22 +1100,22 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
           <t>Health Choice Arizona</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Health Choice Arizona</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>01/28/2026</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -1221,22 +1221,22 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>01/09/2026</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -1340,22 +1340,22 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>01/09/2026</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -1459,22 +1459,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>Banner University Family Care / ACC (AHCCS Complete Care)</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Banner University Family Care / ACC (AHCCS Complete Care)</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>01/21/2026</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -1574,22 +1574,22 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>01/22/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Mercy Care Plan (AHCCCS) - Complete Care &amp; Long Term Care (LTC)</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>01/22/2026</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1683,22 +1683,22 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>01/22/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Mercy Care Plan (AHCCCS) - Complete Care &amp; Long Term Care (LTC)</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>01/22/2026</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1800,22 +1800,22 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>01/28/2026</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -1915,22 +1915,22 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>01/06/2026</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -2028,22 +2028,22 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -2145,22 +2145,22 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -2262,22 +2262,22 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>01/09/2026</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -2375,22 +2375,22 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>01/09/2026</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -2488,22 +2488,22 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
+          <t>01/14/2026</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
           <t>Optum Care Medical Network of Arizona, Utah, &amp; Washington (LifePrint)</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Optum Care Medical Network of Arizona, Utah, &amp; Washington (LifePrint)</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>01/14/2026</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -2601,22 +2601,22 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>01/21/2026</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -2718,22 +2718,22 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>01/21/2026</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -2839,22 +2839,22 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
+          <t>01/22/2026</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
           <t>TRIADA GAP BENEFITS</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>TRIADA GAP BENEFITS</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>01/22/2026</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -2958,22 +2958,22 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
+          <t>01/27/2026</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>01/27/2026</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -3075,22 +3075,22 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
+          <t>01/27/2026</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>01/27/2026</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -3192,22 +3192,22 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
+          <t>01/27/2026</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
           <t>Optum Care Medical Network of Arizona, Utah, &amp; Washington (LifePrint)</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Optum Care Medical Network of Arizona, Utah, &amp; Washington (LifePrint)</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>01/27/2026</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -3309,22 +3309,22 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>LIEN 05</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>01/29/2026</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -3426,22 +3426,22 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
+          <t>01/14/2026</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
           <t>TRIWEST VA CCN CLAIMS</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>TRIWEST VA CCN CLAIMS</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>01/14/2026</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -3539,22 +3539,22 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
+          <t>01/14/2026</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
           <t>TRIWEST VA CCN CLAIMS</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>TRIWEST VA CCN CLAIMS</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>01/14/2026</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -3652,22 +3652,22 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
+          <t>01/23/2026</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
           <t>Medica Health Plan Solutions (Mayo Plan - CHI Health)</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Medica Health Plan Solutions (Mayo Plan - CHI Health)</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>01/23/2026</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -3759,22 +3759,22 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
+          <t>01/23/2026</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
           <t>Medica Health Plan Solutions (Mayo Plan - CHI Health)</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Medica Health Plan Solutions (Mayo Plan - CHI Health)</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>01/23/2026</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -3895,10 +3895,10 @@
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
@@ -3950,22 +3950,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Date of Service</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Responsible Payer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Primary Payer Name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Secondary Payer Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Date of Service</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -4112,22 +4112,22 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>CIGNA MEDICARE SUPPLEMENT INSURANCE</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>01/09/2026</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -4233,22 +4233,22 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Tricare for Life (All Regions)</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>01/09/2026</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -4350,22 +4350,22 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>AARP United Healthcare</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -4471,22 +4471,22 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -4592,22 +4592,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>DME Region D</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Bankers Life Colonial Penn Life</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>01/29/2026</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -4721,22 +4721,22 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>Tricare for Life (All Regions)</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Humana</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Tricare for Life (All Regions)</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -4856,22 +4856,22 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>Mercy Care Plan (AHCCCS) - Complete Care &amp; Long Term Care (LTC)</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Allwell - All States (Centene)</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Mercy Care Plan (AHCCCS) - Complete Care &amp; Long Term Care (LTC)</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -5012,10 +5012,10 @@
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
@@ -5067,22 +5067,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Date of Service</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Responsible Payer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Primary Payer Name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Secondary Payer Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Date of Service</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -5233,22 +5233,22 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -5364,22 +5364,22 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -5491,22 +5491,22 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -5614,22 +5614,22 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -5749,22 +5749,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -5876,22 +5876,22 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -6003,22 +6003,22 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -6134,22 +6134,22 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
           <t>Aetna Senior Supplemental (AESSI) - Secondary Only 62118</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Aetna Senior Supplemental (AESSI) - Secondary Only 62118</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -6261,22 +6261,22 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -6388,22 +6388,22 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -6523,22 +6523,22 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -6662,22 +6662,22 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -6797,22 +6797,22 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -6928,22 +6928,22 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -7059,22 +7059,22 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Unicare Life and Health Insurance (Anthem)</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -7190,22 +7190,22 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -7329,22 +7329,22 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -7464,22 +7464,22 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -7599,22 +7599,22 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -7730,22 +7730,22 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -7861,22 +7861,22 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -7992,22 +7992,22 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>COMBINED INSURANCE CO OF AMERICA</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -8119,22 +8119,22 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
           <t>Bankers Life Colonial Penn Life</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>Bankers Life Colonial Penn Life</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -8250,22 +8250,22 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
           <t>Bankers Life Colonial Penn Life</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>Bankers Life Colonial Penn Life</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -8381,22 +8381,22 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
           <t>Bankers Life Colonial Penn Life</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>Bankers Life Colonial Penn Life</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -8516,22 +8516,22 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
           <t>Bankers Life Colonial Penn Life</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>Bankers Life Colonial Penn Life</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -8655,22 +8655,22 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
           <t>Bankers Life Colonial Penn Life</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>Bankers Life Colonial Penn Life</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -8786,22 +8786,22 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
           <t>Bankers Life Colonial Penn Life</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>Bankers Life Colonial Penn Life</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -8917,22 +8917,22 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
           <t>AARP United Healthcare</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>AARP United Healthcare</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -9052,22 +9052,22 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
           <t>AARP United Healthcare</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>AARP United Healthcare</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -9187,22 +9187,22 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
           <t>AARP United Healthcare</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>Medicare Part B Arizona *</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>AARP United Healthcare</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -9314,22 +9314,22 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -9447,22 +9447,22 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -9576,22 +9576,22 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
@@ -9701,22 +9701,22 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -9830,22 +9830,22 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -9959,22 +9959,22 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
@@ -10084,22 +10084,22 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -10217,22 +10217,22 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
@@ -10346,22 +10346,22 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="H41" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -10471,22 +10471,22 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="G42" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="H42" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
@@ -10600,22 +10600,22 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="H43" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -10729,22 +10729,22 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="H44" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
@@ -10862,22 +10862,22 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
           <t>Aetna Medicare PPO</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>Aetna Medicare PPO</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -10991,22 +10991,22 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
           <t>Aetna Medicare PPO</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="G46" s="5" t="inlineStr">
         <is>
           <t>Aetna Medicare PPO</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="H46" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
@@ -11116,22 +11116,22 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
           <t>Aetna Medicare PPO</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>Aetna Medicare PPO</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="H47" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
@@ -11249,22 +11249,22 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="G48" s="5" t="inlineStr">
         <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="H48" s="5" t="inlineStr">
         <is>
           <t>Arizona Complete Health (Centene)</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
@@ -11368,22 +11368,22 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>Arizona Complete Health (Centene)</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
@@ -11483,22 +11483,22 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="G50" s="5" t="inlineStr">
         <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr">
+      <c r="H50" s="5" t="inlineStr">
         <is>
           <t>Arizona Complete Health (Centene)</t>
-        </is>
-      </c>
-      <c r="H50" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
@@ -11598,22 +11598,22 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="H51" s="5" t="inlineStr">
         <is>
           <t>Arizona Complete Health (Centene)</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
@@ -11717,22 +11717,22 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="G52" s="5" t="inlineStr">
         <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="H52" s="5" t="inlineStr">
         <is>
           <t>Arizona Complete Health (Centene)</t>
-        </is>
-      </c>
-      <c r="H52" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
@@ -11840,22 +11840,22 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
         <is>
           <t>Arizona Complete Health (Centene)</t>
-        </is>
-      </c>
-      <c r="H53" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
@@ -11963,22 +11963,22 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>UMR Wausau / UHIS</t>
         </is>
       </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>Arizona Complete Health (Centene)</t>
-        </is>
-      </c>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
@@ -12111,10 +12111,10 @@
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
@@ -12166,22 +12166,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Date of Service</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Responsible Payer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Primary Payer Name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Secondary Payer Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Date of Service</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -12328,22 +12328,22 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
+          <t>01/15/2026</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
           <t>Arizona Priority Care Plus</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Arizona Priority Care Plus</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>01/15/2026</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -12445,22 +12445,22 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
           <t>CIGNA</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>CIGNA</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>01/09/2026</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -12566,22 +12566,22 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
           <t>UnitedHealthcare Community Plan / Arizona Long Term Care</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>UnitedHealthcare Community Plan / Arizona Long Term Care</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>01/09/2026</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -12681,22 +12681,22 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>01/13/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>UnitedHealthcare Community Plan / Arizona Long Term Care</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>UnitedHealthcare Community Plan / Arizona Long Term Care</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>01/13/2026</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -12798,22 +12798,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>01/14/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>01/14/2026</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -12919,22 +12919,22 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>01/23/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>United Healthcare</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>01/23/2026</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -13042,22 +13042,22 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>01/23/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Blue Cross Blue Shield of Arizona (BCBS AZ)</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>01/23/2026</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -13159,22 +13159,22 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
+          <t>01/23/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
           <t>Gold Kidney Health Plan</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Gold Kidney Health Plan</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>01/23/2026</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -13278,22 +13278,22 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
+          <t>01/23/2026</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
           <t>Gold Kidney Health Plan</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Gold Kidney Health Plan</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>01/23/2026</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -13401,22 +13401,22 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
+          <t>01/26/2026</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
           <t>Tricare West</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Tricare West</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -13545,10 +13545,10 @@
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
@@ -13600,22 +13600,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Date of Service</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Responsible Payer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Primary Payer Name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Secondary Payer Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Date of Service</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -13766,22 +13766,22 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
+          <t>01/08/2026</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Humana Gold Plus HMO</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -13883,22 +13883,22 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>01/08/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
           <t>Optum Care Medical Network of Arizona, Utah, &amp; Washington (LifePrint)</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Optum Care Medical Network of Arizona, Utah, &amp; Washington (LifePrint)</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -14004,22 +14004,22 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
+          <t>01/13/2026</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
           <t>Cigna Medicare Advantage</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Cigna Medicare Advantage</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>01/13/2026</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -14121,22 +14121,22 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>01/14/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>Cigna Medicare Advantage</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Cigna Medicare Advantage</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>01/14/2026</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -14246,22 +14246,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>01/15/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>01/15/2026</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -14367,22 +14367,22 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>HealthSpring Medicare Advantage</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>HealthSpring Medicare Advantage</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>01/21/2026</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -14484,22 +14484,22 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>United Healthcare</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>No Payer</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>01/29/2026</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Show Processed Date and Date Worked 1 as MM/DD/YYYY
Switches both hand-filled date columns from DD/MM/YYYY to MM/DD/YYYY, so
every date in these files now reads in the same order as the source data and
the ambiguity of two conventions in one row is gone. The 13 Processed Dates
seeded from the Notes now display exactly as the Notes wrote them.

Values and row order are unchanged - this is a number format change only.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J8rYoF6JmCLXfVMQM34p4x
</commit_message>
<xml_diff>
--- a/Specialty Claims 2026-S1/2026-01 January - Specialty Claims.xlsx
+++ b/Specialty Claims 2026-S1/2026-01 January - Specialty Claims.xlsx
@@ -27,10 +27,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="MM/DD/YYYY"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="MM/DD/YYYY"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -127,7 +126,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -282,12 +281,12 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Date the claim was processed, shown DD/MM/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date the claim was processed, shown MM/DD/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in.</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Date you worked this claim, shown DD/MM/YYYY. Blank for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date you worked this claim, shown MM/DD/YYYY. Blank for you to fill in.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -332,12 +331,12 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Date the claim was processed, shown DD/MM/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date the claim was processed, shown MM/DD/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in.</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Date you worked this claim, shown DD/MM/YYYY. Blank for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date you worked this claim, shown MM/DD/YYYY. Blank for you to fill in.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -382,12 +381,12 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Date the claim was processed, shown DD/MM/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date the claim was processed, shown MM/DD/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in.</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Date you worked this claim, shown DD/MM/YYYY. Blank for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date you worked this claim, shown MM/DD/YYYY. Blank for you to fill in.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -432,12 +431,12 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Date the claim was processed, shown DD/MM/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date the claim was processed, shown MM/DD/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in.</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Date you worked this claim, shown DD/MM/YYYY. Blank for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date you worked this claim, shown MM/DD/YYYY. Blank for you to fill in.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -482,12 +481,12 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Date the claim was processed, shown DD/MM/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date the claim was processed, shown MM/DD/YYYY. Pre-filled where a Note recorded one; blank otherwise for you to fill in.</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Date you worked this claim, shown DD/MM/YYYY. Blank for you to fill in. Type it the way your Excel expects dates - the cell displays DD/MM/YYYY however it was entered.</t>
+        <t>Date you worked this claim, shown MM/DD/YYYY. Blank for you to fill in.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -15014,7 +15013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -15154,7 +15153,7 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Example of the expected format - Claim Status: "Denied";  Notes: "Corrected service line 1 - resubmitted";  Processed Date: "25/06/2026";  Date Worked 1: "12/08/2026".</t>
+          <t>Example of the expected format - Claim Status: "Denied";  Notes: "Corrected service line 1 - resubmitted";  Processed Date: "06/25/2026";  Date Worked 1: "08/12/2026".</t>
         </is>
       </c>
     </row>
@@ -15171,46 +15170,39 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Both are real dates displayed DD/MM/YYYY. Processed Date is already filled in on the 13 claim lines whose Notes recorded one - the Note still carries the original wording, so nothing was lost. Date Worked 1 starts empty.</t>
+          <t>Both are real dates displayed MM/DD/YYYY, the same order as every other date column in these files and as the source data. Processed Date is already filled in on the 13 claim lines whose Notes recorded one - the Note still carries the original wording, so nothing was lost. Date Worked 1 starts empty.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>Careful when typing into them: Excel reads what you type using its own date setting, not the DD/MM/YYYY the cell displays. On a US Excel, typing 06/25/2026 gives 25 June and the cell then shows 25/06/2026. Type the date the way your Excel expects it and let the cell do the formatting, or check the formula bar afterwards. Every other date column in these files is MM/DD/YYYY, as in the source data.</t>
-        </is>
-      </c>
+      <c r="A26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr"/>
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>How this file feeds the master</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>How this file feeds the master</t>
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>'ALL Claims 2026-S1 - Master.xlsx' (same folder) holds all 1,086 claim lines for 2026 S1. Its Claim Status and Notes columns are formulas that read this file, so anything you type in columns A and B here shows up there. Keep both files in the same folder, keep the file name unchanged, and save this file before opening the master.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>'ALL Claims 2026-S1 - Master.xlsx' (same folder) holds all 1,086 claim lines for 2026 S1. Its Claim Status and Notes columns are formulas that read this file, so anything you type in columns A and B here shows up there. Keep both files in the same folder, keep the file name unchanged, and save this file before opening the master.</t>
+          <t>The link is matched on Line ID (last column), not on row position, so sorting and filtering these sheets is safe. Do not edit or delete the Line ID column, and do not rename the specialty sheet tabs.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>The link is matched on Line ID (last column), not on row position, so sorting and filtering these sheets is safe. Do not edit or delete the Line ID column, and do not rename the specialty sheet tabs.</t>
-        </is>
-      </c>
+      <c r="A30" s="11" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Everything else in this file is a static copy of the source data from 'Specialty Claims Pending 2026-S1.xlsx' (sheet 'Merged').</t>
         </is>

</xml_diff>